<commit_message>
Fehlerbehebung, Tests mit versch Budgetverbesserungen
</commit_message>
<xml_diff>
--- a/Versionen/game_data.xlsx
+++ b/Versionen/game_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\_Privat\Coding\KlimSta\Versionen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1A805BA-8725-40C0-B600-2575E7761FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4930909D-8774-42B0-914D-D221791C8322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="721" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="721" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Massnahmenkarten Spielwerte" sheetId="1" r:id="rId1"/>
@@ -8256,14 +8256,6 @@
       <c r="W73" s="32"/>
       <c r="X73" s="32"/>
       <c r="Y73" s="32"/>
-      <c r="Z73" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA73" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
     </row>
     <row r="74" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="32"/>
@@ -8291,14 +8283,6 @@
       <c r="W74" s="32"/>
       <c r="X74" s="32"/>
       <c r="Y74" s="32"/>
-      <c r="Z74" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA74" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
     </row>
     <row r="75" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="32"/>
@@ -8326,14 +8310,6 @@
       <c r="W75" s="32"/>
       <c r="X75" s="32"/>
       <c r="Y75" s="32"/>
-      <c r="Z75" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA75" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
     </row>
     <row r="76" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="32"/>
@@ -8361,14 +8337,6 @@
       <c r="W76" s="32"/>
       <c r="X76" s="32"/>
       <c r="Y76" s="32"/>
-      <c r="Z76" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA76" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
     </row>
     <row r="77" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="32"/>
@@ -8396,14 +8364,6 @@
       <c r="W77" s="32"/>
       <c r="X77" s="32"/>
       <c r="Y77" s="32"/>
-      <c r="Z77" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA77" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
     </row>
     <row r="78" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="32"/>
@@ -8431,14 +8391,6 @@
       <c r="W78" s="32"/>
       <c r="X78" s="32"/>
       <c r="Y78" s="32"/>
-      <c r="Z78" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA78" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
     </row>
     <row r="79" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="32"/>
@@ -8466,14 +8418,6 @@
       <c r="W79" s="32"/>
       <c r="X79" s="32"/>
       <c r="Y79" s="32"/>
-      <c r="Z79" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA79" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
     </row>
     <row r="80" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="32"/>
@@ -8501,16 +8445,8 @@
       <c r="W80" s="32"/>
       <c r="X80" s="32"/>
       <c r="Y80" s="32"/>
-      <c r="Z80" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA80" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="81" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="32"/>
       <c r="B81" s="80"/>
       <c r="C81" s="40"/>
@@ -8536,16 +8472,8 @@
       <c r="W81" s="32"/>
       <c r="X81" s="32"/>
       <c r="Y81" s="32"/>
-      <c r="Z81" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA81" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="82" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="32"/>
       <c r="B82" s="80"/>
       <c r="C82" s="40"/>
@@ -8571,16 +8499,8 @@
       <c r="W82" s="32"/>
       <c r="X82" s="32"/>
       <c r="Y82" s="32"/>
-      <c r="Z82" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA82" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="83" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="32"/>
       <c r="B83" s="80"/>
       <c r="C83" s="40"/>
@@ -8606,16 +8526,8 @@
       <c r="W83" s="32"/>
       <c r="X83" s="32"/>
       <c r="Y83" s="32"/>
-      <c r="Z83" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA83" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="84" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="84" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="32"/>
       <c r="B84" s="80"/>
       <c r="C84" s="40"/>
@@ -8641,16 +8553,8 @@
       <c r="W84" s="32"/>
       <c r="X84" s="32"/>
       <c r="Y84" s="32"/>
-      <c r="Z84" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA84" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="85" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="32"/>
       <c r="B85" s="80"/>
       <c r="C85" s="40"/>
@@ -8676,16 +8580,8 @@
       <c r="W85" s="32"/>
       <c r="X85" s="32"/>
       <c r="Y85" s="32"/>
-      <c r="Z85" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA85" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="86" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="32"/>
       <c r="B86" s="80"/>
       <c r="C86" s="40"/>
@@ -8711,16 +8607,8 @@
       <c r="W86" s="32"/>
       <c r="X86" s="32"/>
       <c r="Y86" s="32"/>
-      <c r="Z86" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA86" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="87" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="87" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="32"/>
       <c r="B87" s="80"/>
       <c r="C87" s="40"/>
@@ -8746,16 +8634,8 @@
       <c r="W87" s="32"/>
       <c r="X87" s="32"/>
       <c r="Y87" s="32"/>
-      <c r="Z87" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA87" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="88" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="32"/>
       <c r="B88" s="80"/>
       <c r="C88" s="40"/>
@@ -8781,16 +8661,8 @@
       <c r="W88" s="32"/>
       <c r="X88" s="32"/>
       <c r="Y88" s="32"/>
-      <c r="Z88" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA88" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="89" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="32"/>
       <c r="B89" s="80"/>
       <c r="C89" s="40"/>
@@ -8816,16 +8688,8 @@
       <c r="W89" s="32"/>
       <c r="X89" s="32"/>
       <c r="Y89" s="32"/>
-      <c r="Z89" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA89" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="90" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="32"/>
       <c r="B90" s="80"/>
       <c r="C90" s="40"/>
@@ -8851,16 +8715,8 @@
       <c r="W90" s="32"/>
       <c r="X90" s="32"/>
       <c r="Y90" s="32"/>
-      <c r="Z90" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA90" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="91" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="32"/>
       <c r="B91" s="80"/>
       <c r="C91" s="40"/>
@@ -8886,16 +8742,8 @@
       <c r="W91" s="32"/>
       <c r="X91" s="32"/>
       <c r="Y91" s="32"/>
-      <c r="Z91" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA91" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="92" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="32"/>
       <c r="B92" s="80"/>
       <c r="C92" s="40"/>
@@ -8921,16 +8769,8 @@
       <c r="W92" s="32"/>
       <c r="X92" s="32"/>
       <c r="Y92" s="32"/>
-      <c r="Z92" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA92" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="93" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="93" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="32"/>
       <c r="B93" s="80"/>
       <c r="C93" s="40"/>
@@ -8956,16 +8796,8 @@
       <c r="W93" s="32"/>
       <c r="X93" s="32"/>
       <c r="Y93" s="32"/>
-      <c r="Z93" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA93" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="94" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="32"/>
       <c r="B94" s="80"/>
       <c r="C94" s="40"/>
@@ -8991,16 +8823,8 @@
       <c r="W94" s="32"/>
       <c r="X94" s="32"/>
       <c r="Y94" s="32"/>
-      <c r="Z94" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA94" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="95" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="32"/>
       <c r="B95" s="80"/>
       <c r="C95" s="40"/>
@@ -9026,16 +8850,8 @@
       <c r="W95" s="32"/>
       <c r="X95" s="32"/>
       <c r="Y95" s="32"/>
-      <c r="Z95" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA95" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="96" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="32"/>
       <c r="B96" s="80"/>
       <c r="C96" s="40"/>
@@ -9061,16 +8877,8 @@
       <c r="W96" s="32"/>
       <c r="X96" s="32"/>
       <c r="Y96" s="32"/>
-      <c r="Z96" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA96" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="97" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="97" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="32"/>
       <c r="B97" s="80"/>
       <c r="C97" s="40"/>
@@ -9096,16 +8904,8 @@
       <c r="W97" s="32"/>
       <c r="X97" s="32"/>
       <c r="Y97" s="32"/>
-      <c r="Z97" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA97" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="98" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="32"/>
       <c r="B98" s="80"/>
       <c r="C98" s="40"/>
@@ -9131,16 +8931,8 @@
       <c r="W98" s="32"/>
       <c r="X98" s="32"/>
       <c r="Y98" s="32"/>
-      <c r="Z98" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA98" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="99" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="99" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="32"/>
       <c r="B99" s="80"/>
       <c r="C99" s="40"/>
@@ -9166,16 +8958,8 @@
       <c r="W99" s="32"/>
       <c r="X99" s="32"/>
       <c r="Y99" s="32"/>
-      <c r="Z99" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA99" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="100" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="100" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="32"/>
       <c r="B100" s="80"/>
       <c r="C100" s="40"/>
@@ -9201,16 +8985,8 @@
       <c r="W100" s="32"/>
       <c r="X100" s="32"/>
       <c r="Y100" s="32"/>
-      <c r="Z100" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="AA100" t="e">
-        <f>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="101" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="101" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="32"/>
       <c r="B101" s="80"/>
       <c r="C101" s="40"/>
@@ -9237,7 +9013,7 @@
       <c r="X101" s="32"/>
       <c r="Y101" s="32"/>
     </row>
-    <row r="102" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="32"/>
       <c r="B102" s="80"/>
       <c r="C102" s="40"/>
@@ -9264,7 +9040,7 @@
       <c r="X102" s="32"/>
       <c r="Y102" s="32"/>
     </row>
-    <row r="103" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="32"/>
       <c r="B103" s="80"/>
       <c r="C103" s="40"/>
@@ -9291,7 +9067,7 @@
       <c r="X103" s="32"/>
       <c r="Y103" s="32"/>
     </row>
-    <row r="104" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="32"/>
       <c r="B104" s="80"/>
       <c r="C104" s="40"/>
@@ -9318,7 +9094,7 @@
       <c r="X104" s="32"/>
       <c r="Y104" s="32"/>
     </row>
-    <row r="105" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="32"/>
       <c r="B105" s="80"/>
       <c r="C105" s="40"/>
@@ -9345,7 +9121,7 @@
       <c r="X105" s="32"/>
       <c r="Y105" s="32"/>
     </row>
-    <row r="106" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="32"/>
       <c r="B106" s="80"/>
       <c r="C106" s="40"/>
@@ -9372,7 +9148,7 @@
       <c r="X106" s="32"/>
       <c r="Y106" s="32"/>
     </row>
-    <row r="107" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="32"/>
       <c r="B107" s="80"/>
       <c r="C107" s="40"/>
@@ -9399,7 +9175,7 @@
       <c r="X107" s="32"/>
       <c r="Y107" s="32"/>
     </row>
-    <row r="108" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="32"/>
       <c r="B108" s="80"/>
       <c r="C108" s="40"/>
@@ -9426,7 +9202,7 @@
       <c r="X108" s="32"/>
       <c r="Y108" s="32"/>
     </row>
-    <row r="109" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="32"/>
       <c r="B109" s="80"/>
       <c r="C109" s="40"/>
@@ -9453,7 +9229,7 @@
       <c r="X109" s="32"/>
       <c r="Y109" s="32"/>
     </row>
-    <row r="110" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="32"/>
       <c r="B110" s="80"/>
       <c r="C110" s="40"/>
@@ -9480,7 +9256,7 @@
       <c r="X110" s="32"/>
       <c r="Y110" s="32"/>
     </row>
-    <row r="111" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="32"/>
       <c r="B111" s="80"/>
       <c r="C111" s="40"/>
@@ -9507,7 +9283,7 @@
       <c r="X111" s="32"/>
       <c r="Y111" s="32"/>
     </row>
-    <row r="112" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:25" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="32"/>
       <c r="B112" s="80"/>
       <c r="C112" s="40"/>

</xml_diff>